<commit_message>
update cross citation matrices and computation helpers
</commit_message>
<xml_diff>
--- a/datasets/interconnections/bibtex_mapping_of_ids.xlsx
+++ b/datasets/interconnections/bibtex_mapping_of_ids.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonas Hummel\Documents\Studium - PhD Informatik\Survey Paper Interaction\earXplore\interconnections_datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\Documents\Studium - PhD Informatik\Survey Paper Interaction\earXplore\datasets\interconnections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF424723-8D8D-4BAE-82BD-A5C630EE0EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9F8E175-0E38-46EF-8CD9-08B6ED5FC516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1845" yWindow="-20985" windowWidth="16455" windowHeight="19350" xr2:uid="{F5FF20EA-3020-426A-B866-254E9E26798A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F5FF20EA-3020-426A-B866-254E9E26798A}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
   <si>
     <t>ID</t>
   </si>
@@ -1184,21 +1184,6 @@
 	month = sep,
 	year = {2021},
 	pages = {165--170},
-}</t>
-  </si>
-  <si>
-    <t>inproceedings{ID612_gruebler_measurement_2010,
-	title = {Measurement of distal {EMG} signals using a wearable device for reading facial expressions},
-	url = {https://ieeexplore.ieee.org/abstract/document/5626504},
-	doi = {10.1109/IEMBS.2010.5626504},
-	urldate = {2024-12-18},
-	booktitle = {2010 {Annual} {International} {Conference} of the {IEEE} {Engineering} in {Medicine} and {Biology}},
-	author = {Gruebler, Anna and Suzuki, Kenji},
-	month = aug,
-	year = {2010},
-	note = {ISSN: 1558-4615},
-	keywords = {Electrodes, Face, Face recognition, Muscles, Correlation, Electromyography, Humans},
-	pages = {4594--4597},
 }</t>
   </si>
   <si>
@@ -1435,21 +1420,6 @@
 }</t>
   </si>
   <si>
-    <t>inproceedings{ID512_song_facelistener_2022,
-	title = {{FaceListener}: {Recognizing} {Human} {Facial} {Expressions} via {Acoustic} {Sensing} on {Commodity} {Headphones}},
-	shorttitle = {{FaceListener}},
-	url = {https://ieeexplore.ieee.org/document/9825944},
-	doi = {10.1109/IPSN54338.2022.00019},
-	urldate = {2024-12-09},
-	booktitle = {2022 21st {ACM}/{IEEE} {International} {Conference} on {Information} {Processing} in {Sensor} {Networks} ({IPSN})},
-	author = {Song, Xingzhe and Huang, Kai and Gao, Wei},
-	month = may,
-	year = {2022},
-	keywords = {Headphones, Acoustics, Skin, Face recognition, Muscles, Acoustic Sensing, Face Skin Deformation, Headphone, Human Facial Expressions, Knowledge Distillation, Machine learning, Transforms},
-	pages = {145--157},
-}</t>
-  </si>
-  <si>
     <t>article{ID296_rateau_leveraging_2022,
 	title = {Leveraging {Smartwatch} and {Earbuds} {Gesture} {Capture} to {Support} {Wearable} {Interaction}},
 	volume = {6},
@@ -1728,22 +1698,6 @@
 }</t>
   </si>
   <si>
-    <t>inproceedings{ID516_zhu_char_2023,
-	title = {{CHAR}: {Composite} {Head}-body {Activities} {Recognition} with {A} {Single} {Earable} {Device}},
-	shorttitle = {{CHAR}},
-	url = {https://ieeexplore.ieee.org/document/10099218},
-	doi = {10.1109/PERCOM56429.2023.10099218},
-	urldate = {2024-12-16},
-	booktitle = {2023 {IEEE} {International} {Conference} on {Pervasive} {Computing} and {Communications} ({PerCom})},
-	author = {Zhu, Peizhao and Zou, Yongpan and Li, Wenyuan and Wu, Kaishun},
-	month = mar,
-	year = {2023},
-	note = {ISSN: 2474-249X},
-	keywords = {Headphones, Prototypes, Performance evaluation, Legged locomotion, Activity recognition, Composite activity recognition, Earable device, Multi-task learning, Multitasking, Pervasive computing},
-	pages = {212--221},
-}</t>
-  </si>
-  <si>
     <t>inproceedings{ID346_dong_rehearsse_2024,
 	address = {New York, NY, USA},
 	series = {{CHI} '24},
@@ -1866,24 +1820,6 @@
 }</t>
   </si>
   <si>
-    <t>inproceedings{ID291_shojaeifard_left_2024,
-	address = {New York, NY, USA},
-	series = {{IoT} '23},
-	title = {Left or right? {Detecting} driver's head movement on the road},
-	isbn = {979-8-4007-0854-1},
-	shorttitle = {Left or right?},
-	url = {https://dl.acm.org/doi/10.1145/3627050.3627067},
-	doi = {10.1145/3627050.3627067},
-	urldate = {2024-12-19},
-	booktitle = {Proceedings of the 13th {International} {Conference} on the {Internet} of {Things}},
-	publisher = {Association for Computing Machinery},
-	author = {Shojaeifard, Leyla and Islam, Adnanul and Shaheen, Hassan and Schroderus, Vappu and Peltonen, Ella},
-	month = mar,
-	year = {2024},
-	pages = {90--97},
-}</t>
-  </si>
-  <si>
     <t>inproceedings{ID640_srivastava_unvoiced_2024,
 	address = {New York, NY, USA},
 	series = {{SenSys} '24},
@@ -1899,22 +1835,6 @@
 	month = nov,
 	year = {2024},
 	pages = {784--798},
-}</t>
-  </si>
-  <si>
-    <t>article{ID275_shimon_exploring_2024,
-	title = {Exploring {Uni}-manual {Around} {Ear} {Off}-{Device} {Gestures} for {Earables}},
-	volume = {8},
-	url = {https://dl.acm.org/doi/10.1145/3643513},
-	doi = {10.1145/3643513},
-	number = {1},
-	urldate = {2024-10-08},
-	journal = {Proc. ACM Interact. Mob. Wearable Ubiquitous Technol.},
-	author = {Shimon, Shaikh Shawon Arefin and Neshati, Ali and Sun, Junwei and Xu, Qiang and Zhao, Jian},
-	month = mar,
-	year = {2024},
-	note = {Number: 1},
-	pages = {3:1--3:29},
 }</t>
   </si>
   <si>
@@ -2071,6 +1991,492 @@
 	note = {Conference Name: IEEE Transactions on Neural Systems and Rehabilitation Engineering},
 	keywords = {Human computer interaction, Sensors, EMG signals, Muscles, silent command recognition, Transfer learning, Adaptation models, Biological system modeling, Biosensors, user adaptation},
 	pages = {133--143},
+}</t>
+  </si>
+  <si>
+    <t>incollection{jeong_human_2011,
+	address = {Berlin, Heidelberg},
+	title = {Human {Neck}’s {Posture} {Measurement} using a 3-{Axis} {Accelerometer} {Sensor}},
+	volume = {6786},
+	isbn = {978-3-642-21933-7 978-3-642-21934-4},
+	url = {http://link.springer.com/10.1007/978-3-642-21934-4_9},
+	doi = {10.1007/978-3-642-21934-4_9},
+	language = {en},
+	urldate = {2026-04-17},
+	booktitle = {Computational {Science} and {Its} {Applications} - {ICCSA} 2011},
+	publisher = {Springer Berlin Heidelberg},
+	author = {Jeong, Soonmook and Song, Taehoun and Kim, Hyungmin and Kang, Miyoung and Kwon, Keyho and Jeon, Jae Wook},
+	year = {2011},
+	pages = {96--109},
+}</t>
+  </si>
+  <si>
+    <t>incollection{tessendorf_automatic_2012,
+	address = {Berlin, Heidelberg},
+	title = {Automatic {Power}-{Off} for {Binaural} {Hearing} {Instruments}},
+	volume = {7683},
+	isbn = {978-3-642-34897-6 978-3-642-34898-3},
+	url = {http://link.springer.com/10.1007/978-3-642-34898-3_35},
+	doi = {10.1007/978-3-642-34898-3_35},
+	urldate = {2026-04-17},
+	booktitle = {Ambient {Intelligence}},
+	publisher = {Springer Berlin Heidelberg},
+	author = {Tessendorf, Bernd and Derleth, Peter and Feilner, Manuela and Roggen, Daniel and Stiefmeier, Thomas and Tröster, Gerhard},
+	year = {2012},
+	note = {Series Title: Lecture Notes in Computer Science},
+	pages = {409--414},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+incollection{tessendorf_improving_2012,
+	address = {Berlin, Heidelberg},
+	title = {Improving {Game} {Accessibility} with {Vibrotactile}-{Enhanced} {Hearing} {Instruments}},
+	volume = {7382},
+	isbn = {978-3-642-31521-3 978-3-642-31522-0},
+	url = {http://link.springer.com/10.1007/978-3-642-31522-0_70},
+	doi = {10.1007/978-3-642-31522-0_70},
+	urldate = {2026-04-17},
+	booktitle = {Computers {Helping} {People} with {Special} {Needs}},
+	publisher = {Springer Berlin Heidelberg},
+	author = {Tessendorf, Bernd and Derleth, Peter and Feilner, Manuela and Roggen, Daniel and Stiefmeier, Thomas and Tröster, Gerhard},
+	year = {2012},
+	note = {Series Title: Lecture Notes in Computer Science},
+	pages = {463--470},
+}</t>
+  </si>
+  <si>
+    <t>inproceedings{curran_passthoughts_2016,
+	title = {Passthoughts authentication with low cost {EarEEG}},
+	issn = {1558-4615},
+	url = {https://ieeexplore.ieee.org/abstract/document/7591112},
+	doi = {10.1109/EMBC.2016.7591112},
+	urldate = {2026-04-17},
+	booktitle = {2016 38th {Annual} {International} {Conference} of the {IEEE} {Engineering} in {Medicine} and {Biology} {Society} ({EMBC})},
+	author = {Curran, Max T. and Yang, Jong-kai and Merrill, Nick and Chuang, John},
+	month = aug,
+	year = {2016},
+	keywords = {Ear, Electrodes, Electroencephalography, Authentication, Sensors, Face, Testing},
+	pages = {1979--1982},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inproceedings{favre-felix_real-time_2017,
+	title = {Real-time estimation of eye gaze by in-ear electrodes},
+	issn = {1558-4615},
+	url = {https://ieeexplore.ieee.org/document/8037754},
+	doi = {10.1109/EMBC.2017.8037754},
+	urldate = {2026-04-17},
+	booktitle = {2017 39th {Annual} {International} {Conference} of the {IEEE} {Engineering} in {Medicine} and {Biology} {Society} ({EMBC})},
+	author = {Favre-Félix, A. and Graversen, C. and Dau, T. and Lunner, T.},
+	month = jul,
+	year = {2017},
+	note = {ISSN: 1558-4615},
+	keywords = {Band-pass filters, Correlation, Ear, Electrodes, Electrooculography, Hearing aids, Real-time systems},
+	pages = {4086--4089},
+}
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+@inproceedings{cheah_wearable_2018,
+	address = {Funchal, Madeira, Portugal},
+	title = {A {Wearable} {Silent} {Speech} {Interface} based on {Magnetic} {Sensors} with {Motion}-{Artefact} {Removal}:},
+	isbn = {978-989-758-307-0},
+	url = {https://www.scitepress.org/DigitalLibrary/Link.aspx?doi=10.5220/0006573200560062},
+	doi = {10.5220/0006573200560062},
+	language = {en},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 11th {International} {Joint} {Conference} on {Biomedical} {Engineering} {Systems} and {Technologies}},
+	publisher = {SCITEPRESS - Science and Technology Publications},
+	author = {Cheah, Lam A. and Gilbert, James M. and Gonzalez, Jose A. and Green, Phil D. and R. Ell, Stephen and K. Moore, Roger and Holdsworth, Ed},
+	year = {2018},
+	pages = {56--62},
+}</t>
+  </si>
+  <si>
+    <t>inproceedings{ID626_ma_oesense_2021,
+	address = {New York, NY, USA},
+	series = {{MobiSys} '21},
+	title = {{OESense}: employing occlusion effect for in-ear human sensing},
+	isbn = {978-1-4503-8443-8},
+	shorttitle = {{OESense}},
+	url = {https://dl.acm.org/doi/10.1145/3458864.3467680},
+	doi = {10.1145/3458864.3467680},
+	urldate = {2024-12-18},
+	booktitle = {Proceedings of the 19th {Annual} {International} {Conference} on {Mobile} {Systems}, {Applications}, and {Services}},
+	publisher = {Association for Computing Machinery},
+	author = {Ma, Dong and Ferlini, Andrea and Mascolo, Cecilia},
+	month = jun,
+	year = {2021},
+	pages = {175--187},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{ID512_song_facelistener_2022,
+	title = {{FaceListener}: {Recognizing} {Human} {Facial} {Expressions} via {Acoustic} {Sensing} on {Commodity} {Headphones}},
+	shorttitle = {{FaceListener}},
+	url = {https://ieeexplore.ieee.org/document/9825944},
+	doi = {10.1109/IPSN54338.2022.00019},
+	urldate = {2024-12-09},
+	booktitle = {2022 21st {ACM}/{IEEE} {International} {Conference} on {Information} {Processing} in {Sensor} {Networks} ({IPSN})},
+	author = {Song, Xingzhe and Huang, Kai and Gao, Wei},
+	month = may,
+	year = {2022},
+	keywords = {Headphones, Acoustics, Skin, Face recognition, Muscles, Acoustic Sensing, Face Skin Deformation, Headphone, Human Facial Expressions, Knowledge Distillation, Machine learning, Transforms},
+	pages = {145--157},
+}</t>
+  </si>
+  <si>
+    <t>inproceedings{iguma_input_2023,
+	address = {New York, NY, USA},
+	series = {{ISWC} '23},
+	title = {Input {Interface} with {Touch} and {Non}-touch {Interactions} using {Atmospheric} {Pressure} for {Hearable} {Devices}},
+	isbn = {979-8-4007-0199-3},
+	url = {https://dl.acm.org/doi/10.1145/3594738.3611354},
+	doi = {10.1145/3594738.3611354},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 2023 {ACM} {International} {Symposium} on {Wearable} {Computers}},
+	publisher = {Association for Computing Machinery},
+	author = {Iguma, Koki and Murao, Kazuya and Watanabe, Hiroki},
+	month = oct,
+	year = {2023},
+	pages = {1--5},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+article{ID275_shimon_exploring_2024,
+	title = {Exploring {Uni}-manual {Around} {Ear} {Off}-{Device} {Gestures} for {Earables}},
+	volume = {8},
+	url = {https://dl.acm.org/doi/10.1145/3643513},
+	doi = {10.1145/3643513},
+	number = {1},
+	urldate = {2024-10-08},
+	journal = {Proc. ACM Interact. Mob. Wearable Ubiquitous Technol.},
+	author = {Shimon, Shaikh Shawon Arefin and Neshati, Ali and Sun, Junwei and Xu, Qiang and Zhao, Jian},
+	month = mar,
+	year = {2024},
+	note = {Number: 1},
+	pages = {3:1--3:29},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{ID291_shojaeifard_left_2024,
+	address = {New York, NY, USA},
+	series = {{IoT} '23},
+	title = {Left or right? {Detecting} driver's head movement on the road},
+	isbn = {979-8-4007-0854-1},
+	shorttitle = {Left or right?},
+	url = {https://dl.acm.org/doi/10.1145/3627050.3627067},
+	doi = {10.1145/3627050.3627067},
+	urldate = {2024-12-19},
+	booktitle = {Proceedings of the 13th {International} {Conference} on the {Internet} of {Things}},
+	publisher = {Association for Computing Machinery},
+	author = {Shojaeifard, Leyla and Islam, Adnanul and Shaheen, Hassan and Schroderus, Vappu and Peltonen, Ella},
+	month = mar,
+	year = {2024},
+	pages = {90--97},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{amesaka_flexear-tips_2025,
+	address = {New York, NY, USA},
+	series = {{CHI} '25},
+	title = {{FlexEar}-{Tips}: {Shape}-{Adjustable} {Ear} {Tips} {Using} {Pressure} {Control}},
+	isbn = {979-8-4007-1394-1},
+	shorttitle = {{FlexEar}-{Tips}},
+	url = {https://dl.acm.org/doi/10.1145/3706598.3714177},
+	doi = {10.1145/3706598.3714177},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 2025 {CHI} {Conference} on {Human} {Factors} in {Computing} {Systems}},
+	publisher = {Association for Computing Machinery},
+	author = {Amesaka, Takashi and Yamamoto, Takumi and Watanabe, Hiroki and Shizuki, Buntarou and Sugiura, Yuta},
+	month = apr,
+	year = {2025},
+	pages = {1--13},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{chugh_unlocking_2025,
+	title = {Unlocking {Eye} {Gestures} with {Earable} {Inertial} {Sensing} for {Accessible} {HCI}},
+	issn = {2155-2509},
+	url = {https://ieeexplore.ieee.org/abstract/document/10885707},
+	doi = {10.1109/COMSNETS63942.2025.10885707},
+	urldate = {2026-04-17},
+	booktitle = {2025 17th {International} {Conference} on {COMmunication} {Systems} and {NETworks} ({COMSNETS})},
+	author = {Chugh, Garvit and Chakraborty, Suchetana and Chakraborty, Sandip},
+	month = jan,
+	year = {2025},
+	pages = {828--832},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+article{gao_trumpet_2025,
+	title = {The {Trumpet} of the {Swan}: {Decoding} {Lip} {Language} for {Speech}-impaired {Users} through {COTS} {Earbuds}},
+	volume = {9},
+	shorttitle = {The {Trumpet} of the {Swan}},
+	url = {https://dl.acm.org/doi/10.1145/3770648},
+	doi = {10.1145/3770648},
+	number = {4},
+	urldate = {2026-04-17},
+	journal = {Proc. ACM Interact. Mob. Wearable Ubiquitous Technol.},
+	author = {Gao, Ming and Dai, Yichen and Zhou, Zhanbo and Guo, Zhengxin and Han, Jinsong and Xiao, Fu},
+	month = dec,
+	year = {2025},
+	pages = {175:1--175:32},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{kang_earpressure_2025,
+	address = {New York, NY, USA},
+	series = {{UIST} '25},
+	title = {{EarPressure} {VR}: {Ear} {Canal} {Pressure} {Feedback} for {Enhancing} {Environmental} {Presence} in {Virtual} {Reality}},
+	isbn = {979-8-4007-2037-6},
+	url = {https://dl.acm.org/doi/10.1145/3746059.3747618},
+	doi = {10.1145/3746059.3747618},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 38th {Annual} {ACM} {Symposium} on {User} {Interface} {Software} and {Technology}},
+	publisher = {Association for Computing Machinery},
+	author = {Kang, Seongjun and Kim, Gwangbin and Gim, Bocheon and Park, Jeongju and Shin, Semoo and Kim, SeungJun},
+	month = sep,
+	year = {2025},
+	pages = {1--17},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{kim_budsid_2025,
+	address = {Yokohama Japan},
+	title = {{BudsID}: {Mobile}-{Ready} and {Expressive} {Finger} {Identification} {Input} for {Earbuds}},
+	isbn = {979-8-4007-1394-1},
+	shorttitle = {{BudsID}},
+	url = {https://dl.acm.org/doi/10.1145/3706598.3714133},
+	doi = {10.1145/3706598.3714133},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 2025 {CHI} {Conference} on {Human} {Factors} in {Computing} {Systems}},
+	publisher = {ACM},
+	author = {Kim, Jiwan and Han, Mingyu and Oakley, Ian},
+	month = apr,
+	year = {2025},
+	pages = {1--17},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+article{liu_eareog_2025,
+	title = {{EarEOG}: {Using} {Headphones} and {Around}-the-{Ear} {EOG} {Signals} for {Real}-{Time} {Wheelchair} {Control}},
+	volume = {9},
+	shorttitle = {{EarEOG}},
+	url = {https://dl.acm.org/doi/10.1145/3725833},
+	doi = {10.1145/3725833},
+	number = {3},
+	urldate = {2026-04-17},
+	journal = {Proc. ACM Hum.-Comput. Interact.},
+	author = {Liu, Peichen and Puthusserypady, Sadasivan and MacKenzie, I. Scott and Uyanik, Cihan and Hansen, John Paulin},
+	month = may,
+	year = {2025},
+	pages = {ETRA08:1--ETRA08:16},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+article{tang_wireless_2025,
+	title = {Wireless {Silent} {Speech} {Interface} {Using} {Multichannel} {Textile} {EMG} {Sensors} {Integrated} {Into} {Headphones}},
+	volume = {74},
+	issn = {1557-9662},
+	url = {https://ieeexplore.ieee.org/abstract/document/11052721},
+	doi = {10.1109/TIM.2025.3583386},
+	urldate = {2026-04-17},
+	journal = {IEEE Transactions on Instrumentation and Measurement},
+	author = {Tang, Chenyu and Mallah, Josée and Kazieczko, Dominika and Yi, Wentian and Kandukuri, Tharun Reddy and Occhipinti, Edoardo and Mishra, Bhaskar and Mehta, Sunita and Occhipinti, Luigi G.},
+	year = {2025},
+	pages = {1--10},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{yang_leakyfeeder_2025,
+	address = {New York, NY, USA},
+	series = {{SenSys} '25},
+	title = {{LeakyFeeder}: {In}-{Air} {Gesture} {Control} {Through} {Leaky} {Acoustic} {Waves}},
+	isbn = {979-8-4007-1479-5},
+	url = {https://dl.acm.org/doi/10.1145/3715014.3722054},
+	doi = {10.1145/3715014.3722054},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 23rd {ACM} {Conference} on {Embedded} {Networked} {Sensor} {Systems}},
+	publisher = {Association for Computing Machinery},
+	author = {Yang, Yongjie and Chen, Tao and An, Zhenlin and Cao, Shirui and Fan, Xiaoran and Shangguan, Longfei},
+	month = may,
+	year = {2025},
+	pages = {144--157},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+@inproceedings{zhao_palatetouch_2025,
+	address = {New York, NY, USA},
+	series = {{CHI} '25},
+	title = {{PalateTouch} : {Enabling} {Palate} as a {Touchpad} to {Interact} with {Earphones} {Using} {Acoustic} {Sensing}},
+	isbn = {979-8-4007-1394-1},
+	url = {https://dl.acm.org/doi/10.1145/3706598.3713211},
+	doi = {10.1145/3706598.3713211},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 2025 {CHI} {Conference} on {Human} {Factors} in {Computing} {Systems}},
+	publisher = {Association for Computing Machinery},
+	author = {Zhao, Yankai and Zhang, Jin and Li, Jiao and Sun, Tao},
+	month = apr,
+	year = {2025},
+	pages = {1--22},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+@article{zhu_char_2025,
+	title = {{CHAR}: {Composite} {Head}-{Body} {Activities} {Recognition} {With} a {Single} {Earable} {Device}},
+	volume = {24},
+	issn = {1558-0660},
+	shorttitle = {{CHAR}},
+	url = {https://ieeexplore.ieee.org/abstract/document/10916516},
+	doi = {10.1109/TMC.2025.3548647},
+	number = {7},
+	urldate = {2026-04-17},
+	journal = {IEEE Transactions on Mobile Computing},
+	author = {Zhu, Peizhao and Zhu, Yuzheng and Li, Wenyuan and He, Yanbo and Zou, Yongpan and Wu, Kaishun and Leung, Victor C. M.},
+	month = jul,
+	year = {2025},
+	pages = {6532--6549},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{zitz_heatables_2025,
+	address = {New York, NY, USA},
+	series = {{ISWC} '25},
+	title = {Heatables: {Effects} of {Infrared}-{LED}-{Induced} {Ear} {Heating} on {Thermal} {Perception}, {Comfort}, and {Cognitive} {Performance}},
+	isbn = {979-8-4007-1481-8},
+	url = {https://dl.acm.org/doi/10.1145/3715071.3750421},
+	doi = {10.1145/3715071.3750421},
+	urldate = {2026-04-17},
+	booktitle = {Proceedings of the 2025 {ACM} {International} {Symposium} on {Wearable} {Computers}},
+	publisher = {Association for Computing Machinery},
+	author = {Zitz, Valeria and Küttner, Michael and Hummel, Jonas and Knierim, Michael T. and Beigl, Michael and Röddiger, Tobias},
+	month = oct,
+	year = {2025},
+	pages = {91--97},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+incollection{Bodsworth_ear_2026,
+	address = {Cham},
+	title = {Ear {Haptics}: {A} {Preliminary} {Suitability} {Study} of a {Novel} {Auricular} {Haptic} {Human}-{Machine} {Interface}},
+	volume = {16334},
+	isbn = {978-3-032-12391-6 978-3-032-12392-3},
+	shorttitle = {Ear {Haptics}},
+	url = {https://link.springer.com/10.1007/978-3-032-12392-3_23},
+	doi = {10.1007/978-3-032-12392-3_23},
+	urldate = {2026-04-17},
+	booktitle = {{HCI} {International} 2025 – {Late} {Breaking} {Papers}},
+	publisher = {Springer Nature Switzerland},
+	author = {Bodsworth, Chris and Blundell, James and Birrell, Stewart and Payre, William},
+	year = {2026},
+	pages = {345--363},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{dong_poster_2026,
+	address = {New York, NY, USA},
+	series = {{UbiComp} {Companion} '25},
+	title = {Poster: {Recognizing} {Hidden}-in-the-{Ear} {Private} {Key} for {Reliable} {Silent} {Speech} {Interface} {Using} {Multi}-{Task} {Learning}},
+	isbn = {979-8-4007-1477-1},
+	url = {https://dl.acm.org/doi/10.1145/3714394.3754429},
+	doi = {10.1145/3714394.3754429},
+	urldate = {2026-04-17},
+	booktitle = {Companion of the 2025 {ACM} {International} {Joint} {Conference} on {Pervasive} and {Ubiquitous} {Computing}},
+	publisher = {Association for Computing Machinery},
+	author = {Dong, Xuefu and Xu, Liqiang and He, Lixing and Han, Zengyi and Christofferson, Kenneth and Chen, Yifei and Taya, Akihito and Nishiyama, Yuuki and Sezaki, Kaoru},
+	month = dec,
+	year = {2026},
+	pages = {211--215},
+}</t>
+  </si>
+  <si>
+    <t>article{liu_eareog_2025,
+	title = {{EarEOG}: {Using} {Headphones} and {Around}-the-{Ear} {EOG} {Signals} for {Real}-{Time} {Wheelchair} {Control}},
+	volume = {9},
+	shorttitle = {{EarEOG}},
+	url = {https://dl.acm.org/doi/10.1145/3725833},
+	doi = {10.1145/3725833},
+	number = {3},
+	urldate = {2026-04-17},
+	journal = {Proc. ACM Hum.-Comput. Interact.},
+	author = {Liu, Peichen and Puthusserypady, Sadasivan and MacKenzie, I. Scott and Uyanik, Cihan and Hansen, John Paulin},
+	month = may,
+	year = {2025},
+	pages = {ETRA08:1--ETRA08:16},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+article{takaki_headgaze_2026,
+	title = {{HeadGaze}: {Natural} {Gaze} {Estimation} {While} {Walking} {From} a {Single} {IMU} on {Earbuds}},
+	volume = {26},
+	issn = {1558-1748},
+	shorttitle = {{HeadGaze}},
+	url = {https://ieeexplore.ieee.org/abstract/document/11391500},
+	doi = {10.1109/JSEN.2026.3661116},
+	number = {6},
+	urldate = {2026-04-17},
+	journal = {IEEE Sensors Journal},
+	author = {Takaki, Ken and Kamezaki, Mitsuhiro and Sasatani, Takuya and Murakami, Hiroaki and Kawahara, Yoshihiro},
+	month = mar,
+	year = {2026},
+	pages = {8849--8863},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{van_oort_earmag_2026,
+	address = {New York, NY, USA},
+	series = {{UbiComp} {Companion} '25},
+	title = {{EarMag}: {In}-{Ear} {Magnetosensing} for {Jaw} and {Head} {Gesture}-{Based} {Human}-{Computer} {Interaction}},
+	isbn = {979-8-4007-1477-1},
+	shorttitle = {{EarMag}},
+	url = {https://dl.acm.org/doi/10.1145/3714394.3757254},
+	doi = {10.1145/3714394.3757254},
+	urldate = {2026-04-17},
+	booktitle = {Companion of the 2025 {ACM} {International} {Joint} {Conference} on {Pervasive} and {Ubiquitous} {Computing}},
+	publisher = {Association for Computing Machinery},
+	author = {van Oort, Max J. F. and Sáenz, Gabriel E. and Tirtajana, Selina and Pawełczak, Przemysław},
+	month = dec,
+	year = {2026},
+	pages = {834--840},
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+inproceedings{yuma_mouth_2026,
+	address = {New York, NY, USA},
+	series = {{UbiComp} {Companion} '25},
+	title = {Mouth {Gesture} {Recognition} {Using} {PPG} {Sensors} in {Earbuds}},
+	isbn = {979-8-4007-1477-1},
+	url = {https://dl.acm.org/doi/10.1145/3714394.3756205},
+	doi = {10.1145/3714394.3756205},
+	urldate = {2026-04-17},
+	booktitle = {Companion of the 2025 {ACM} {International} {Joint} {Conference} on {Pervasive} and {Ubiquitous} {Computing}},
+	publisher = {Association for Computing Machinery},
+	author = {Yuma, Taiki and Murao, Kazuya},
+	month = dec,
+	year = {2026},
+	pages = {1024--1030},
 }</t>
   </si>
 </sst>
@@ -2130,8 +2536,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{15F3F71E-5F14-4F36-BD12-EF8DBC22420E}" name="Tabelle1" displayName="Tabelle1" ref="A1:B119" totalsRowShown="0">
-  <autoFilter ref="A1:B119" xr:uid="{15F3F71E-5F14-4F36-BD12-EF8DBC22420E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{15F3F71E-5F14-4F36-BD12-EF8DBC22420E}" name="Tabelle1" displayName="Tabelle1" ref="A1:B142" totalsRowShown="0">
+  <autoFilter ref="A1:B142" xr:uid="{15F3F71E-5F14-4F36-BD12-EF8DBC22420E}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D99C8DB6-12A6-4AA3-8098-FFEF06F78696}" name="ID"/>
     <tableColumn id="2" xr3:uid="{477576D2-543C-4CD2-8FBA-133065FAB206}" name="Bibtex"/>
@@ -2457,13 +2863,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D024FC-F189-4140-BB6D-32424F58D85E}">
-  <dimension ref="A1:B119"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:B142"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="121.4609375" customWidth="1"/>
+    <col min="2" max="2" width="121.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2471,7 +2877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="131.15" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2479,7 +2885,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2487,7 +2893,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2495,7 +2901,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2503,7 +2909,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2511,7 +2917,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2519,7 +2925,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2527,7 +2933,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2535,884 +2941,1068 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="102" x14ac:dyDescent="0.4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="72.900000000000006" x14ac:dyDescent="0.4">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="262.3" x14ac:dyDescent="0.4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="261" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="189.45" x14ac:dyDescent="0.4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="174.9" x14ac:dyDescent="0.4">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="306" x14ac:dyDescent="0.4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="262.3" x14ac:dyDescent="0.4">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="174" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="261" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="306" x14ac:dyDescent="0.4">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="276.89999999999998" x14ac:dyDescent="0.4">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="276.89999999999998" x14ac:dyDescent="0.4">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="189.45" x14ac:dyDescent="0.4">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" ht="262.3" x14ac:dyDescent="0.4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="262.3" x14ac:dyDescent="0.4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="291.45" x14ac:dyDescent="0.4">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="261" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="261" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" ht="290" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" ht="276.89999999999998" x14ac:dyDescent="0.4">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" ht="262.3" x14ac:dyDescent="0.4">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" ht="262.3" x14ac:dyDescent="0.4">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" ht="189.45" x14ac:dyDescent="0.4">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="261" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" ht="261" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>113</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" ht="262.3" x14ac:dyDescent="0.4">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>114</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" ht="204" x14ac:dyDescent="0.4">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>115</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" ht="218.6" x14ac:dyDescent="0.4">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" ht="233.15" x14ac:dyDescent="0.4">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>117</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" ht="247.75" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="232" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>118</v>
       </c>
       <c r="B119" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" ht="203" x14ac:dyDescent="0.35">
+      <c r="A120">
         <v>119</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" ht="261" x14ac:dyDescent="0.35">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" ht="203" x14ac:dyDescent="0.35">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="203" x14ac:dyDescent="0.35">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" ht="203" x14ac:dyDescent="0.35">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" ht="232" x14ac:dyDescent="0.35">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>